<commit_message>
actualizar documentacion sobre enrutamiento
</commit_message>
<xml_diff>
--- a/docs/routing.xlsx
+++ b/docs/routing.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EducacionIT\Documents\networks\CISCO\saves\ccna3-mj19\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F79F2AB-2B8E-4A4C-8FEC-5568D3D0961F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26104494-ABC1-4F53-9E7C-7E6A377112E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{9775BEA3-CF6A-4BD0-98D3-A009A1CC9C91}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{9775BEA3-CF6A-4BD0-98D3-A009A1CC9C91}"/>
   </bookViews>
   <sheets>
     <sheet name="route" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="136">
   <si>
     <t>10.0.0.0/8</t>
   </si>
@@ -66,9 +66,6 @@
   </si>
   <si>
     <t>10.0.0.0/30</t>
-  </si>
-  <si>
-    <t>NETWORK\PACKET</t>
   </si>
   <si>
     <t>10.54.11.20</t>
@@ -625,6 +622,127 @@
   </si>
   <si>
     <t>255.255.0.0</t>
+  </si>
+  <si>
+    <t>Direccion</t>
+  </si>
+  <si>
+    <t>Ceros Izq.</t>
+  </si>
+  <si>
+    <t>Resultado</t>
+  </si>
+  <si>
+    <t>ACAD</t>
+  </si>
+  <si>
+    <t>0DB8</t>
+  </si>
+  <si>
+    <t>0001</t>
+  </si>
+  <si>
+    <t>0000</t>
+  </si>
+  <si>
+    <t>2001</t>
+  </si>
+  <si>
+    <t>DB8</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>::</t>
+  </si>
+  <si>
+    <t>Conjunto</t>
+  </si>
+  <si>
+    <t>2001:DB8:ACAD:1::1/64</t>
+  </si>
+  <si>
+    <t>Global Address</t>
+  </si>
+  <si>
+    <t>Interface ID</t>
+  </si>
+  <si>
+    <t>SnetId</t>
+  </si>
+  <si>
+    <t>Prefix</t>
+  </si>
+  <si>
+    <t>64</t>
+  </si>
+  <si>
+    <t>EUI-64</t>
+  </si>
+  <si>
+    <t>D3</t>
+  </si>
+  <si>
+    <t>D1</t>
+  </si>
+  <si>
+    <t>9B</t>
+  </si>
+  <si>
+    <t>FF</t>
+  </si>
+  <si>
+    <t>FE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4D </t>
+  </si>
+  <si>
+    <t>link</t>
+  </si>
+  <si>
+    <t>16b</t>
+  </si>
+  <si>
+    <t>!7b</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">FE80::D19B:58FF:FE19:134D </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>LINK-LOCAL</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">MAC-ADDRESS:  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="0"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>D39B.5819.134D</t>
+    </r>
+  </si>
+  <si>
+    <t>NET\PACKET</t>
   </si>
 </sst>
 </file>
@@ -633,9 +751,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -674,6 +792,14 @@
     <font>
       <sz val="11"/>
       <color rgb="FFC00000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -723,7 +849,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -896,33 +1022,119 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color theme="1"/>
+      </top>
+      <bottom style="medium">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -933,101 +1145,130 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1371,269 +1612,269 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F929431-7726-4028-A622-641A837AF0E9}">
   <dimension ref="A1:H10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="8" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1" s="49" t="s">
         <v>9</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" s="49" t="s">
         <v>10</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" s="49" t="s">
         <v>11</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" s="49" t="s">
         <v>12</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" s="49" t="s">
         <v>13</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" s="49" t="s">
         <v>14</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" s="49" t="s">
         <v>15</v>
       </c>
-      <c r="H1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="51" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="B2" s="73" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="74" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" s="74" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" s="74" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" s="74" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" s="74" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" s="74" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="45" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="B3" s="75" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="76" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" s="76" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" s="76" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="76" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="76" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" s="76" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="44" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="B4" s="75" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="77" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" s="76" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" s="76" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" s="76" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" s="76" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" s="76" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="B5" s="75" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="75" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="76" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" s="76" t="s">
+        <v>17</v>
+      </c>
+      <c r="F5" s="76" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" s="76" t="s">
+        <v>17</v>
+      </c>
+      <c r="H5" s="76" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="B6" s="75" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="75" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" s="77" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" s="76" t="s">
+        <v>17</v>
+      </c>
+      <c r="F6" s="76" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" s="76" t="s">
+        <v>17</v>
+      </c>
+      <c r="H6" s="76" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="45" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="B7" s="75" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="75" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" s="75" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="77" t="s">
+        <v>17</v>
+      </c>
+      <c r="F7" s="77" t="s">
+        <v>17</v>
+      </c>
+      <c r="G7" s="76" t="s">
+        <v>17</v>
+      </c>
+      <c r="H7" s="76" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="44" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="B8" s="75" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="75" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8" s="75" t="s">
+        <v>16</v>
+      </c>
+      <c r="E8" s="75" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" s="75" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" s="77" t="s">
+        <v>17</v>
+      </c>
+      <c r="H8" s="76" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="45" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+      <c r="B9" s="75" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="75" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="75" t="s">
+        <v>16</v>
+      </c>
+      <c r="E9" s="75" t="s">
+        <v>16</v>
+      </c>
+      <c r="F9" s="75" t="s">
+        <v>16</v>
+      </c>
+      <c r="G9" s="75" t="s">
+        <v>16</v>
+      </c>
+      <c r="H9" s="76" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="67" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>18</v>
+      <c r="B10" s="78" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="78" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" s="78" t="s">
+        <v>16</v>
+      </c>
+      <c r="E10" s="78" t="s">
+        <v>16</v>
+      </c>
+      <c r="F10" s="78" t="s">
+        <v>16</v>
+      </c>
+      <c r="G10" s="78" t="s">
+        <v>16</v>
+      </c>
+      <c r="H10" s="79" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -1644,110 +1885,110 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C64266CF-856B-416A-9223-968A84079862}">
   <dimension ref="A1:B14"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" t="s">
         <v>19</v>
       </c>
-      <c r="B1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>31</v>
-      </c>
-      <c r="B5" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>21</v>
-      </c>
-      <c r="B7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>22</v>
       </c>
       <c r="B8">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B9">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B10">
         <v>90</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B11">
         <v>110</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B12">
         <v>115</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B13">
         <v>120</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B14">
         <v>255</v>
@@ -1761,296 +2002,296 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE8565DC-3EF5-4EBD-A9E2-63F501E9451D}">
   <dimension ref="A1:M8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.77734375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="5" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="6.44140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="5.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="32" t="s">
+        <v>82</v>
+      </c>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="32" t="s">
+        <v>85</v>
+      </c>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="34"/>
+      <c r="J1" s="32" t="s">
+        <v>82</v>
+      </c>
+      <c r="K1" s="33"/>
+      <c r="L1" s="33"/>
+      <c r="M1" s="34"/>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="I2" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="J2" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="M2" s="9" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="K1" s="13"/>
-      <c r="L1" s="13"/>
-      <c r="M1" s="14"/>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A2" s="7" t="s">
+      <c r="B3" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="B2" s="15" t="s">
-        <v>84</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="E2" s="16" t="s">
-        <v>58</v>
-      </c>
-      <c r="F2" s="15" t="s">
-        <v>84</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="I2" s="16" t="s">
-        <v>58</v>
-      </c>
-      <c r="J2" s="15" t="s">
-        <v>98</v>
-      </c>
-      <c r="K2" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="L2" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="M2" s="16" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A3" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="B3" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="C3" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="D3" s="19">
+      <c r="C3" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" s="12">
         <v>127255255255</v>
       </c>
-      <c r="E3" s="20" t="s">
-        <v>50</v>
-      </c>
-      <c r="F3" s="28" t="s">
-        <v>89</v>
-      </c>
-      <c r="G3" s="29" t="s">
-        <v>93</v>
-      </c>
-      <c r="H3" s="30">
+      <c r="E3" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="F3" s="18" t="s">
+        <v>88</v>
+      </c>
+      <c r="G3" s="19" t="s">
+        <v>92</v>
+      </c>
+      <c r="H3" s="20">
         <v>10255255255</v>
       </c>
-      <c r="I3" s="31" t="s">
-        <v>93</v>
-      </c>
-      <c r="J3" s="17" t="s">
-        <v>103</v>
-      </c>
-      <c r="K3" s="43">
+      <c r="I3" s="21" t="s">
+        <v>92</v>
+      </c>
+      <c r="J3" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="K3" s="28">
         <v>8</v>
       </c>
-      <c r="L3" s="19">
+      <c r="L3" s="12">
         <v>1</v>
       </c>
-      <c r="M3" s="44">
+      <c r="M3" s="29">
         <f>2^(32-K3)-2</f>
         <v>16777214</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="B4" s="21" t="s">
-        <v>41</v>
-      </c>
-      <c r="C4" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="D4" s="23">
+    <row r="4" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="D4" s="16">
         <v>191255255255</v>
       </c>
-      <c r="E4" s="24" t="s">
-        <v>51</v>
-      </c>
-      <c r="F4" s="32" t="s">
-        <v>90</v>
-      </c>
-      <c r="G4" s="33" t="s">
+      <c r="E4" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="F4" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="G4" s="23" t="s">
+        <v>93</v>
+      </c>
+      <c r="H4" s="24" t="s">
+        <v>91</v>
+      </c>
+      <c r="I4" s="25" t="s">
         <v>94</v>
       </c>
-      <c r="H4" s="34" t="s">
-        <v>92</v>
-      </c>
-      <c r="I4" s="35" t="s">
-        <v>95</v>
-      </c>
-      <c r="J4" s="21" t="s">
-        <v>104</v>
-      </c>
-      <c r="K4" s="45">
-        <v>16</v>
-      </c>
-      <c r="L4" s="23">
-        <v>16</v>
-      </c>
-      <c r="M4" s="46">
+      <c r="J4" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="K4" s="30">
+        <v>16</v>
+      </c>
+      <c r="L4" s="16">
+        <v>16</v>
+      </c>
+      <c r="M4" s="31">
         <f t="shared" ref="M4:M5" si="0">2^(32-K4)-2</f>
         <v>65534</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A5" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="B5" s="17" t="s">
-        <v>42</v>
-      </c>
-      <c r="C5" s="18" t="s">
-        <v>47</v>
-      </c>
-      <c r="D5" s="19">
+    <row r="5" spans="1:13" ht="45" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D5" s="12">
         <v>223255255255</v>
       </c>
-      <c r="E5" s="20" t="s">
-        <v>52</v>
-      </c>
-      <c r="F5" s="28" t="s">
-        <v>91</v>
-      </c>
-      <c r="G5" s="36" t="s">
-        <v>97</v>
-      </c>
-      <c r="H5" s="30">
+      <c r="E5" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="F5" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="G5" s="26" t="s">
+        <v>96</v>
+      </c>
+      <c r="H5" s="20">
         <v>192168255255</v>
       </c>
-      <c r="I5" s="37" t="s">
-        <v>96</v>
-      </c>
-      <c r="J5" s="17" t="s">
-        <v>102</v>
-      </c>
-      <c r="K5" s="43">
+      <c r="I5" s="27" t="s">
+        <v>95</v>
+      </c>
+      <c r="J5" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="K5" s="28">
         <v>24</v>
       </c>
-      <c r="L5" s="19">
+      <c r="L5" s="12">
         <v>256</v>
       </c>
-      <c r="M5" s="44">
+      <c r="M5" s="29">
         <f t="shared" si="0"/>
         <v>254</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A6" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="B6" s="21" t="s">
-        <v>43</v>
-      </c>
-      <c r="C6" s="22" t="s">
-        <v>48</v>
-      </c>
-      <c r="D6" s="23">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="D6" s="16">
         <v>239255255255</v>
       </c>
-      <c r="E6" s="24" t="s">
-        <v>53</v>
+      <c r="E6" s="17" t="s">
+        <v>52</v>
       </c>
       <c r="F6" s="38" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G6" s="39"/>
       <c r="H6" s="39"/>
       <c r="I6" s="40"/>
       <c r="J6" s="38" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="K6" s="39"/>
       <c r="L6" s="39"/>
       <c r="M6" s="40"/>
     </row>
-    <row r="7" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="B7" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="C7" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="D7" s="19">
+    <row r="7" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="D7" s="12">
         <v>255255255255</v>
       </c>
-      <c r="E7" s="20" t="s">
-        <v>54</v>
+      <c r="E7" s="13" t="s">
+        <v>53</v>
       </c>
       <c r="F7" s="41" t="s">
-        <v>88</v>
-      </c>
-      <c r="G7" s="10"/>
-      <c r="H7" s="10"/>
-      <c r="I7" s="42"/>
+        <v>87</v>
+      </c>
+      <c r="G7" s="42"/>
+      <c r="H7" s="42"/>
+      <c r="I7" s="43"/>
       <c r="J7" s="41" t="s">
-        <v>88</v>
-      </c>
-      <c r="K7" s="10"/>
-      <c r="L7" s="10"/>
-      <c r="M7" s="42"/>
-    </row>
-    <row r="8" spans="1:13" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="B8" s="25">
+        <v>87</v>
+      </c>
+      <c r="K7" s="42"/>
+      <c r="L7" s="42"/>
+      <c r="M7" s="43"/>
+    </row>
+    <row r="8" spans="1:13" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="B8" s="35">
         <f>2^32</f>
         <v>4294967296</v>
       </c>
-      <c r="C8" s="26"/>
-      <c r="D8" s="26"/>
-      <c r="E8" s="27"/>
-      <c r="F8" s="25">
+      <c r="C8" s="36"/>
+      <c r="D8" s="36"/>
+      <c r="E8" s="37"/>
+      <c r="F8" s="35">
         <f>2^32</f>
         <v>4294967296</v>
       </c>
-      <c r="G8" s="26"/>
-      <c r="H8" s="26"/>
-      <c r="I8" s="27"/>
-      <c r="J8" s="25">
+      <c r="G8" s="36"/>
+      <c r="H8" s="36"/>
+      <c r="I8" s="37"/>
+      <c r="J8" s="35">
         <f>2^32</f>
         <v>4294967296</v>
       </c>
-      <c r="K8" s="26"/>
-      <c r="L8" s="26"/>
-      <c r="M8" s="27"/>
+      <c r="K8" s="36"/>
+      <c r="L8" s="36"/>
+      <c r="M8" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -2071,116 +2312,349 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DE3A49A-43BB-415B-ABDB-844C12E64EE1}">
-  <dimension ref="A1:F5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:Q10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="3" width="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.77734375" style="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="10" width="7" customWidth="1"/>
+    <col min="11" max="11" width="2.7109375" customWidth="1"/>
+    <col min="12" max="12" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="5.42578125" style="47" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="5.28515625" style="47" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="4.85546875" style="47" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="19.7109375" style="48" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B1" s="64" t="s">
+        <v>118</v>
+      </c>
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
+      <c r="E1" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="F1" s="64" t="s">
+        <v>119</v>
+      </c>
+      <c r="G1" s="64"/>
+      <c r="H1" s="64"/>
+      <c r="I1" s="64"/>
+      <c r="J1" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="M1" s="49" t="s">
+        <v>54</v>
+      </c>
+      <c r="N1" s="49" t="s">
+        <v>55</v>
+      </c>
+      <c r="O1" s="49" t="s">
+        <v>63</v>
+      </c>
+      <c r="P1" s="50" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A2" s="51" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="54">
+        <v>2001</v>
+      </c>
+      <c r="C2" s="54" t="s">
+        <v>108</v>
+      </c>
+      <c r="D2" s="54" t="s">
+        <v>107</v>
+      </c>
+      <c r="E2" s="54" t="s">
+        <v>109</v>
+      </c>
+      <c r="F2" s="54" t="s">
+        <v>110</v>
+      </c>
+      <c r="G2" s="54" t="s">
+        <v>110</v>
+      </c>
+      <c r="H2" s="54" t="s">
+        <v>110</v>
+      </c>
+      <c r="I2" s="54" t="s">
+        <v>109</v>
+      </c>
+      <c r="J2" s="54" t="s">
+        <v>122</v>
+      </c>
+      <c r="L2" s="51" t="s">
         <v>59</v>
       </c>
-      <c r="B1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C1" t="s">
-        <v>56</v>
-      </c>
-      <c r="D1" t="s">
-        <v>64</v>
-      </c>
-      <c r="E1" s="5" t="s">
+      <c r="M2" s="52">
+        <v>2000</v>
+      </c>
+      <c r="N2" s="52" t="s">
         <v>65</v>
       </c>
-      <c r="F1" t="s">
+      <c r="O2" s="53">
+        <v>3</v>
+      </c>
+      <c r="P2" s="54" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q2" s="51" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A3" s="45" t="s">
+        <v>105</v>
+      </c>
+      <c r="B3" s="57" t="s">
+        <v>111</v>
+      </c>
+      <c r="C3" s="57" t="s">
+        <v>112</v>
+      </c>
+      <c r="D3" s="57" t="s">
+        <v>107</v>
+      </c>
+      <c r="E3" s="57" t="s">
+        <v>113</v>
+      </c>
+      <c r="F3" s="57" t="s">
+        <v>114</v>
+      </c>
+      <c r="G3" s="57" t="s">
+        <v>114</v>
+      </c>
+      <c r="H3" s="57" t="s">
+        <v>114</v>
+      </c>
+      <c r="I3" s="57" t="s">
+        <v>113</v>
+      </c>
+      <c r="J3" s="57" t="s">
+        <v>122</v>
+      </c>
+      <c r="L3" s="45" t="s">
         <v>60</v>
       </c>
-      <c r="B2">
-        <v>2000</v>
-      </c>
-      <c r="C2" t="s">
-        <v>66</v>
-      </c>
-      <c r="D2">
-        <v>3</v>
-      </c>
-      <c r="E2" s="5" t="s">
+      <c r="M3" s="55" t="s">
         <v>67</v>
       </c>
-      <c r="F2" t="s">
+      <c r="N3" s="55" t="s">
+        <v>73</v>
+      </c>
+      <c r="O3" s="56">
+        <v>7</v>
+      </c>
+      <c r="P3" s="57" t="s">
+        <v>74</v>
+      </c>
+      <c r="Q3" s="45" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A4" s="44" t="s">
+        <v>116</v>
+      </c>
+      <c r="B4" s="60" t="s">
+        <v>111</v>
+      </c>
+      <c r="C4" s="60" t="s">
+        <v>112</v>
+      </c>
+      <c r="D4" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="E4" s="60" t="s">
+        <v>113</v>
+      </c>
+      <c r="F4" s="66" t="s">
+        <v>115</v>
+      </c>
+      <c r="G4" s="66"/>
+      <c r="H4" s="66"/>
+      <c r="I4" s="60" t="s">
+        <v>113</v>
+      </c>
+      <c r="J4" s="60" t="s">
+        <v>122</v>
+      </c>
+      <c r="L4" s="44" t="s">
         <v>61</v>
       </c>
-      <c r="B3" t="s">
+      <c r="M4" s="58" t="s">
         <v>68</v>
       </c>
-      <c r="C3" t="s">
-        <v>74</v>
-      </c>
-      <c r="D3">
-        <v>7</v>
-      </c>
-      <c r="E3" s="5" t="s">
+      <c r="N4" s="58" t="s">
+        <v>72</v>
+      </c>
+      <c r="O4" s="59">
+        <v>10</v>
+      </c>
+      <c r="P4" s="60" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q4" s="44" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="46" t="s">
+        <v>106</v>
+      </c>
+      <c r="B5" s="65" t="s">
+        <v>117</v>
+      </c>
+      <c r="C5" s="65"/>
+      <c r="D5" s="65"/>
+      <c r="E5" s="65"/>
+      <c r="F5" s="65"/>
+      <c r="G5" s="65"/>
+      <c r="H5" s="65"/>
+      <c r="I5" s="65"/>
+      <c r="J5" s="65"/>
+      <c r="L5" s="46" t="s">
+        <v>62</v>
+      </c>
+      <c r="M5" s="61" t="s">
+        <v>69</v>
+      </c>
+      <c r="N5" s="61" t="s">
         <v>75</v>
       </c>
-      <c r="F3" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>62</v>
-      </c>
-      <c r="B4" t="s">
-        <v>69</v>
-      </c>
-      <c r="C4" t="s">
-        <v>73</v>
-      </c>
-      <c r="D4">
-        <v>10</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="F4" t="s">
+      <c r="O5" s="62">
+        <v>8</v>
+      </c>
+      <c r="P5" s="63" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q5" s="46" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>63</v>
-      </c>
-      <c r="B5" t="s">
-        <v>70</v>
-      </c>
-      <c r="C5" t="s">
-        <v>76</v>
-      </c>
-      <c r="D5">
-        <v>8</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="F5" t="s">
-        <v>81</v>
-      </c>
+    <row r="6" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="72" t="s">
+        <v>123</v>
+      </c>
+      <c r="B7" s="64" t="s">
+        <v>134</v>
+      </c>
+      <c r="C7" s="64"/>
+      <c r="D7" s="64"/>
+      <c r="E7" s="64"/>
+      <c r="F7" s="64"/>
+      <c r="G7" s="64"/>
+      <c r="H7" s="64"/>
+      <c r="I7" s="64"/>
+      <c r="J7" s="64"/>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A8" s="69" t="s">
+        <v>131</v>
+      </c>
+      <c r="B8" s="52" t="s">
+        <v>124</v>
+      </c>
+      <c r="C8" s="52" t="s">
+        <v>126</v>
+      </c>
+      <c r="D8" s="52">
+        <v>58</v>
+      </c>
+      <c r="E8" s="52" t="s">
+        <v>127</v>
+      </c>
+      <c r="F8" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="G8" s="52">
+        <v>19</v>
+      </c>
+      <c r="H8" s="52">
+        <v>13</v>
+      </c>
+      <c r="I8" s="52" t="s">
+        <v>129</v>
+      </c>
+      <c r="J8" s="52" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A9" s="70" t="s">
+        <v>132</v>
+      </c>
+      <c r="B9" s="55" t="s">
+        <v>125</v>
+      </c>
+      <c r="C9" s="55" t="s">
+        <v>126</v>
+      </c>
+      <c r="D9" s="55">
+        <v>58</v>
+      </c>
+      <c r="E9" s="55" t="s">
+        <v>127</v>
+      </c>
+      <c r="F9" s="55" t="s">
+        <v>128</v>
+      </c>
+      <c r="G9" s="55">
+        <v>19</v>
+      </c>
+      <c r="H9" s="55">
+        <v>13</v>
+      </c>
+      <c r="I9" s="55" t="s">
+        <v>129</v>
+      </c>
+      <c r="J9" s="55" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="71" t="s">
+        <v>58</v>
+      </c>
+      <c r="B10" s="68" t="s">
+        <v>133</v>
+      </c>
+      <c r="C10" s="68"/>
+      <c r="D10" s="68"/>
+      <c r="E10" s="68"/>
+      <c r="F10" s="68"/>
+      <c r="G10" s="68"/>
+      <c r="H10" s="68"/>
+      <c r="I10" s="68"/>
+      <c r="J10" s="68"/>
     </row>
   </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="B7:J7"/>
+    <mergeCell ref="B10:J10"/>
+    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="F1:I1"/>
+    <mergeCell ref="B5:J5"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="B3:B4 E2:J3 E4 I4:J4" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>